<commit_message>
Publier PARALLAXE v0.2.1 : jeu coopératif, radio et classeur complet
Ajouter le jeu 3D, les trois lieux, 54 anomalies intégrées, les avatars et reflets, le serveur coopératif et la radio WebRTC.
Corriger les activations micro et interface annulées, avec 19 tests radio et 4 tests du contrôleur.
Inclure le classeur de 120 anomalies, les archives PC et sources, le modèle GLB, les guides et la CI.
Les limites de validation GPU, microphone et TURN sont documentées dans docs/QA.md.
</commit_message>
<xml_diff>
--- a/docs/PARALLAXE_Design_Complet.xlsx
+++ b/docs/PARALLAXE_Design_Complet.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthèse" sheetId="1" r:id="R83c7ea82cdde49e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Boucle" sheetId="2" r:id="R87e2aaee61a549bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anomalies" sheetId="3" r:id="Rf6fcc9d2bcc044db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coopération" sheetId="4" r:id="R6e3a01744b3247ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Radio" sheetId="5" r:id="R4b3a049d2c614c5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Personnages" sheetId="6" r:id="R8ea18143cbcc4689"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Niveaux" sheetId="7" r:id="R2c80bd39626e4bd5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lieux" sheetId="8" r:id="R97cf5e5b18ed4911"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Direction artistique" sheetId="9" r:id="R3da3ac57945940aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audio" sheetId="10" r:id="Rcd983a22f1954b00"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Commandes" sheetId="11" r:id="R7077c20af6eb4cd4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Narration" sheetId="12" r:id="R72369e6f05ea470a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="13" r:id="Rf3047eb4c2b642b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA" sheetId="14" r:id="Rd5a82cbf77d1405e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Références" sheetId="15" r:id="Re9ac3f53d5044ed2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthèse" sheetId="1" r:id="Rd860a8f3c5fd43ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Boucle" sheetId="2" r:id="R473a0ffd5eff42af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anomalies" sheetId="3" r:id="R3095c15dee364e1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coopération" sheetId="4" r:id="R2332f36235c94e02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Radio" sheetId="5" r:id="Rc308d49f9a9a4280"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Personnages" sheetId="6" r:id="Re871745b31d14919"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Niveaux" sheetId="7" r:id="R9413597ed0de4b86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lieux" sheetId="8" r:id="R29bca919142a44ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Direction artistique" sheetId="9" r:id="R658864451f604223"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audio" sheetId="10" r:id="R18e419a2df38430c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Commandes" sheetId="11" r:id="Rdc22a7b299c64b73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Narration" sheetId="12" r:id="R4300c79667974324"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="13" r:id="R64f150af41194520"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA" sheetId="14" r:id="R4850e4e2055445f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Références" sheetId="15" r:id="Red9d6b2d8fac4aa9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -713,8 +713,8 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="P9_Production" displayName="P9_Production" ref="A5:H59" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:H59"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="P9_Production" displayName="P9_Production" ref="A5:H61" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:H61"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Priorité"/>
@@ -730,8 +730,8 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="P9_QA" displayName="P9_QA" ref="A5:H81" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:H81"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="P9_QA" displayName="P9_QA" ref="A5:H86" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:H86"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Priorité"/>
@@ -747,8 +747,8 @@
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="P9_References" displayName="P9_References" ref="A5:G31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:G31"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="P9_References" displayName="P9_References" ref="A5:G34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:G34"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Type"/>
@@ -810,8 +810,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="P9_Radio" displayName="P9_Radio" ref="A5:H32" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:H32"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="P9_Radio" displayName="P9_Radio" ref="A5:H35" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:H35"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Système / preuve"/>
@@ -1153,7 +1153,7 @@
     </x:row>
     <x:row r="4" ht="23" customHeight="1">
       <x:c r="A4" s="6" t="str">
-        <x:v>Conception et suivi · édition 0.2.0 · 26 octobre 2026</x:v>
+        <x:v>Conception et suivi · édition 0.2.1 · 26 octobre 2026</x:v>
       </x:c>
       <x:c r="B4" s="3"/>
       <x:c r="C4" s="3"/>
@@ -1204,8 +1204,8 @@
         <x:v>Lots de production</x:v>
       </x:c>
       <x:c r="E7" s="34" t="n">
-        <x:f>COUNTA('Production'!$A$6:$A$59)</x:f>
-        <x:v>54</x:v>
+        <x:f>COUNTA('Production'!$A$6:$A$61)</x:f>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="F7" s="3"/>
       <x:c r="G7" s="3"/>
@@ -1224,8 +1224,8 @@
         <x:v>Lots en code ou présents</x:v>
       </x:c>
       <x:c r="E8" s="34" t="n">
-        <x:f>COUNTIFS('Production'!$E$6:$E$59,"Présent")+COUNTIFS('Production'!$E$6:$E$59,"Implémenté — QA partielle")</x:f>
-        <x:v>27</x:v>
+        <x:f>COUNTIFS('Production'!$E$6:$E$61,"Présent")+COUNTIFS('Production'!$E$6:$E$61,"Implémenté — QA partielle")</x:f>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F8" s="3"/>
       <x:c r="G8" s="3"/>
@@ -1244,7 +1244,7 @@
         <x:v>Lots à vérifier / éprouver</x:v>
       </x:c>
       <x:c r="E9" s="34" t="n">
-        <x:f>COUNTIFS('Production'!$E$6:$E$59,"À vérifier")+COUNTIFS('Production'!$E$6:$E$59,"À exécuter")+COUNTIFS('Production'!$E$6:$E$59,"À tester sur GPU")+COUNTIFS('Production'!$E$6:$E$59,"À tester sur appareils")</x:f>
+        <x:f>COUNTIFS('Production'!$E$6:$E$61,"À vérifier")+COUNTIFS('Production'!$E$6:$E$61,"À exécuter")+COUNTIFS('Production'!$E$6:$E$61,"À tester sur GPU")+COUNTIFS('Production'!$E$6:$E$61,"À tester sur appareils")</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="F9" s="3"/>
@@ -1264,7 +1264,7 @@
         <x:v>Lots futurs</x:v>
       </x:c>
       <x:c r="E10" s="34" t="n">
-        <x:f>COUNTIFS('Production'!$E$6:$E$59,"Conçu — non implémenté")</x:f>
+        <x:f>COUNTIFS('Production'!$E$6:$E$61,"Conçu — non implémenté")</x:f>
         <x:v>17</x:v>
       </x:c>
       <x:c r="F10" s="3"/>
@@ -1284,8 +1284,8 @@
         <x:v>Priorités P0</x:v>
       </x:c>
       <x:c r="E11" s="34" t="n">
-        <x:f>COUNTIFS('Production'!$B$6:$B$59,"P0")</x:f>
-        <x:v>17</x:v>
+        <x:f>COUNTIFS('Production'!$B$6:$B$61,"P0")</x:f>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="F11" s="3"/>
       <x:c r="G11" s="3"/>
@@ -1304,7 +1304,7 @@
         <x:v>Priorités P1</x:v>
       </x:c>
       <x:c r="E12" s="34" t="n">
-        <x:f>COUNTIFS('Production'!$B$6:$B$59,"P1")</x:f>
+        <x:f>COUNTIFS('Production'!$B$6:$B$61,"P1")</x:f>
         <x:v>28</x:v>
       </x:c>
       <x:c r="F12" s="3"/>
@@ -1324,8 +1324,8 @@
         <x:v>Parcours QA documentés</x:v>
       </x:c>
       <x:c r="E13" s="34" t="n">
-        <x:f>COUNTA('QA'!$A$6:$A$81)</x:f>
-        <x:v>76</x:v>
+        <x:f>COUNTA('QA'!$A$6:$A$86)</x:f>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="F13" s="3"/>
       <x:c r="G13" s="3"/>
@@ -1543,7 +1543,7 @@
     </x:row>
     <x:row r="28" ht="31" customHeight="1">
       <x:c r="A28" s="37" t="str">
-        <x:v>Vraie voix avec permission explicite, PTT, six effets de réception et calibration sans micro. Corps articulés et reflets planaires.</x:v>
+        <x:v>Correctif 0.2.1 : flux micro tardifs arrêtés après extinction / sortie ; réactivation récente préservée ; commande de radio débloquée sans attendre une ancienne permission.</x:v>
       </x:c>
       <x:c r="B28" s="37"/>
       <x:c r="C28" s="37"/>
@@ -1555,7 +1555,7 @@
     </x:row>
     <x:row r="29" ht="39" customHeight="1">
       <x:c r="A29" s="37" t="str">
-        <x:v>Vérifié : 17 tests de règles, 12 tests radio, 11 suites CPU 3D et campagne D1 à quatre clients HTTP. Deux onglets échangent offre/réponse, mais zéro candidat ICE empêche la connexion audio. GPU et microphones physiques non éprouvés.</x:v>
+        <x:v>Correctif 0.2.1 : 19 tests radio, 4 du contrôleur UI, deux builds et test portable à deux clients HTTP réussis. Preuves v0.2 conservées : 17 règles, 11 suites CPU 3D et D1 quatre clients. GPU, microphones physiques, transport vocal et TURN réel restent non validés.</x:v>
       </x:c>
       <x:c r="B29" s="37"/>
       <x:c r="C29" s="37"/>
@@ -2160,7 +2160,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3eade47a9daa4217"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb869eebedf0b44f5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2806,7 +2806,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f099ff108a84c6a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R110b77c14b7242b9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3314,7 +3314,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd534c747764e44e5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd05a49a6e2943b6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3495,7 +3495,7 @@
         <x:v>Contenu</x:v>
       </x:c>
       <x:c r="D9" s="11" t="str">
-        <x:v>Intégrer les 54 anomalies présentes au catalogue runtime v0.2.</x:v>
+        <x:v>Intégrer les 54 anomalies présentes au catalogue runtime 0.2.1.</x:v>
       </x:c>
       <x:c r="E9" s="13" t="str">
         <x:v>Implémenté — QA partielle</x:v>
@@ -3663,7 +3663,7 @@
         <x:v>QA15–QA25, QA41–QA46</x:v>
       </x:c>
       <x:c r="H15" s="11" t="str">
-        <x:v>D1 local réel : quatre clients HTTP, neuf consensus concurrents, campagne trois lieux et références propres, signalisation privée et départ réussis. Ni microphones physiques ni trajet TURN réel testés par ce rapport.</x:v>
+        <x:v>Rapport v0.2 conservé : D1 local réel : quatre clients HTTP, neuf consensus concurrents, campagne trois lieux et références propres, signalisation privée et départ réussis. Ni microphones physiques ni trajet TURN réel testés par ce rapport.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="40" customHeight="1">
@@ -4290,7 +4290,7 @@
         <x:v>Un prototype jouable n’est pas une validation commerciale complète.</x:v>
       </x:c>
     </x:row>
-    <x:row r="40" ht="40" customHeight="1">
+    <x:row r="40" ht="64" customHeight="1">
       <x:c r="A40" s="12" t="str">
         <x:v>P35</x:v>
       </x:c>
@@ -4301,7 +4301,7 @@
         <x:v>Export</x:v>
       </x:c>
       <x:c r="D40" s="12" t="str">
-        <x:v>Fournir source, édition autonome, instructions et Excel v0.2 synchronisé.</x:v>
+        <x:v>Fournir source, édition autonome, instructions et Excel 0.2.1 synchronisé.</x:v>
       </x:c>
       <x:c r="E40" s="13" t="str">
         <x:v>À vérifier</x:v>
@@ -4310,10 +4310,10 @@
         <x:v>Livraison</x:v>
       </x:c>
       <x:c r="G40" s="12" t="str">
-        <x:v>Version 0.2.0</x:v>
+        <x:v>Version 0.2.1</x:v>
       </x:c>
       <x:c r="H40" s="12" t="str">
-        <x:v>Dépôt GitHub et archive reproductibles ; aucun secret ou dépendance volumineuse inutile.</x:v>
+        <x:v>Builds local / hébergé et test portable à deux clients HTTP réussis. Classeur synchronisé. Intégrité des nouvelles archives et GitHub CI à vérifier après assemblage / publication ; rapport docs/qa-final-v0.2.1.json.</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="40" customHeight="1">
@@ -4810,20 +4810,72 @@
         <x:v>GLTFExporter puis GLTFLoader réussis ; matériaux de base et articulation rigide explicités. Visuel GPU restant.</x:v>
       </x:c>
     </x:row>
+    <x:row r="60" ht="64" customHeight="1">
+      <x:c r="A60" s="12" t="str">
+        <x:v>P55</x:v>
+      </x:c>
+      <x:c r="B60" s="12" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C60" s="12" t="str">
+        <x:v>Cycle du microphone</x:v>
+      </x:c>
+      <x:c r="D60" s="12" t="str">
+        <x:v>Fermer les flux retournés après extinction / sortie et protéger une réactivation plus récente.</x:v>
+      </x:c>
+      <x:c r="E60" s="13" t="str">
+        <x:v>Implémenté — QA partielle</x:v>
+      </x:c>
+      <x:c r="F60" s="12" t="str">
+        <x:v>Audio / cycle asynchrone</x:v>
+      </x:c>
+      <x:c r="G60" s="12" t="str">
+        <x:v>Radio R28–R29 ; QA77–QA79</x:v>
+      </x:c>
+      <x:c r="H60" s="12" t="str">
+        <x:v>19/19 tests radio réussis, dont 7 nouveaux : extinction, micro seul, anciennes réponses, nouvelle demande et sortie. Avant correction : 6 échecs / 1 succès ; après : 7/7. Pistes et API simulées ; aucun microphone physique ni transmission mesurée.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="77" customHeight="1">
+      <x:c r="A61" s="11" t="str">
+        <x:v>P56</x:v>
+      </x:c>
+      <x:c r="B61" s="11" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C61" s="11" t="str">
+        <x:v>Commande de radio</x:v>
+      </x:c>
+      <x:c r="D61" s="11" t="str">
+        <x:v>Libérer l’état d’attente de l’interface à l’extinction et isoler chaque nouvelle opération.</x:v>
+      </x:c>
+      <x:c r="E61" s="13" t="str">
+        <x:v>Implémenté — QA partielle</x:v>
+      </x:c>
+      <x:c r="F61" s="11" t="str">
+        <x:v>UI / contrôleur</x:v>
+      </x:c>
+      <x:c r="G61" s="11" t="str">
+        <x:v>Radio R30 ; QA80</x:v>
+      </x:c>
+      <x:c r="H61" s="11" t="str">
+        <x:v>4/4 tests de radio-actions : arrêt libère l’attente ; ancienne réponse ignorée, refus courant signalé ; changement de salon / démontage invalide les callbacks ; appel dans le geste utilisateur et échec synchrone nettoyé. Typecheck réussi. Aucun test DOM, micro physique ou GPU.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="E6:E59">
+  <x:conditionalFormatting sqref="E6:E61">
     <x:cfRule type="containsText" dxfId="33" priority="1" operator="containsText" text="Bloqué"/>
     <x:cfRule type="containsText" dxfId="34" priority="2" operator="containsText" text="Validé"/>
     <x:cfRule type="containsText" dxfId="35" priority="3" operator="containsText" text="Réussi"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="E6:E59">
+    <x:dataValidation type="list" sqref="E6:E61">
       <x:formula1>"Présent,Prévu,Implémenté — QA partielle,Validé,À vérifier,Conçu — non implémenté,Bloqué,Réussi,Partiel,À exécuter,À tester sur GPU,À tester sur appareils,Conception définie,Contrôle structurel partiel"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd1f9ee089d5c426d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1cd1f55f13514701"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5839,7 +5891,7 @@
         <x:v>Contrôler IDs, couverture runtime, compteurs, statuts, tableaux et rendu.</x:v>
       </x:c>
       <x:c r="E41" s="11" t="str">
-        <x:v>120 fiches ; 54 en code ; 66 futures ; 15 feuilles ; 76 parcours QA.</x:v>
+        <x:v>120 fiches ; 54 en code ; 66 futures ; 15 feuilles ; 80 parcours QA.</x:v>
       </x:c>
       <x:c r="F41" s="13" t="str">
         <x:v>Réussi</x:v>
@@ -5848,7 +5900,7 @@
         <x:v>Artifact Tool / XLSX</x:v>
       </x:c>
       <x:c r="H41" s="11" t="str">
-        <x:v>Générateur v0.2 : 120 IDs uniques, 54 runtime, 66 prévus ; compteurs et pools recalculés, statuts modifiés puis restaurés ; contrôle du XLSX et rendus représentatifs.</x:v>
+        <x:v>Générateur v0.2.1 : 120 IDs uniques, 54 runtime, 66 prévus ; versions cohérentes, compteurs et pools recalculés, modifications temporaires restaurées et feuilles touchées rendues.</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="40" customHeight="1">
@@ -6111,7 +6163,7 @@
         <x:v>Campagne quatre clients HTTP traversée avec lieux/références synchronisés ; mode unique couvert dans les règles. Vérification graphique multi-appareils restante.</x:v>
       </x:c>
     </x:row>
-    <x:row r="52" ht="51" customHeight="1">
+    <x:row r="52" ht="64" customHeight="1">
       <x:c r="A52" s="12" t="str">
         <x:v>QA47</x:v>
       </x:c>
@@ -6134,7 +6186,7 @@
         <x:v>Chrome / Firefox / Safari</x:v>
       </x:c>
       <x:c r="H52" s="12" t="str">
-        <x:v>Tests avec doubles de périphériques : aucune demande avant action explicite, démarrage muet et libération des pistes. Permission et indicateur sur micro physique non observés.</x:v>
+        <x:v>19 tests radio réussis avec doubles de périphériques : permission explicite, démarrage muet et arrêt des flux reçus après invalidation. Aucun microphone physique ni indicateur matériel observé.</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="51" customHeight="1">
@@ -6238,7 +6290,7 @@
         <x:v>Navigateurs / certificats</x:v>
       </x:c>
       <x:c r="H56" s="12" t="str">
-        <x:v>12 tests radio incluent une origine LAN non sécurisée : indisponibilité technique annoncée, aucun prompt micro ni altération de preuve. Certificat LAN réel non testé.</x:v>
+        <x:v>19 tests radio incluent une origine LAN non sécurisée : indisponibilité technique annoncée, aucun prompt micro ni altération de preuve. Certificat LAN réel non testé.</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="40" customHeight="1">
@@ -6319,7 +6371,7 @@
         <x:v>Les tests établissent l’indépendance de la preuve au consentement et au transport. Scénario complet de coupure pendant une session vocale physique restant.</x:v>
       </x:c>
     </x:row>
-    <x:row r="60" ht="51" customHeight="1">
+    <x:row r="60" ht="64" customHeight="1">
       <x:c r="A60" s="12" t="str">
         <x:v>QA55</x:v>
       </x:c>
@@ -6342,7 +6394,7 @@
         <x:v>WebAudio et inspection code</x:v>
       </x:c>
       <x:c r="H60" s="12" t="str">
-        <x:v>Tests radio : fermeture et instances retirées contrôlées ; états PTT expirent. Vérifier à l’oreille les queues d’effet et transitions répétées sur appareil.</x:v>
+        <x:v>Correctif v0.2.1 : les demandes micro invalidées ne peuvent plus installer un flux tardif ; les pistes reçues sont arrêtées. Nettoyage vérifié avec doubles de périphériques. Queues sonores et matériel restent à écouter.</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="51" customHeight="1">
@@ -6891,20 +6943,150 @@
         <x:v>Deux onglets réels : salon, écoute sans permission micro, calibration écrite et échange offre/réponse réussis ; négociation stable. ICE terminé avec zéro candidat local/distant : liaison audio non établie. Aucun flux vocal ni micro physique validé.</x:v>
       </x:c>
     </x:row>
+    <x:row r="82" ht="64" customHeight="1">
+      <x:c r="A82" s="12" t="str">
+        <x:v>QA77</x:v>
+      </x:c>
+      <x:c r="B82" s="12" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C82" s="12" t="str">
+        <x:v>Permission après arrêt</x:v>
+      </x:c>
+      <x:c r="D82" s="12" t="str">
+        <x:v>Différer getUserMedia, éteindre la radio ou couper le micro seul puis résoudre l’autorisation avec un flux.</x:v>
+      </x:c>
+      <x:c r="E82" s="12" t="str">
+        <x:v>Chaque piste tardive est stoppée ; aucun flux local retenu. L’écoute seule reste active si elle a été conservée.</x:v>
+      </x:c>
+      <x:c r="F82" s="13" t="str">
+        <x:v>Réussi</x:v>
+      </x:c>
+      <x:c r="G82" s="12" t="str">
+        <x:v>Tests radio à promesse différée</x:v>
+      </x:c>
+      <x:c r="H82" s="12" t="str">
+        <x:v>Deux tests réussis : désactiver toute la radio ou le micro seul avant résolution. La piste tardive est stoppée ; le micro reste éteint et l’écoute choisie est conservée. Promesses et flux simulés.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83" ht="64" customHeight="1">
+      <x:c r="A83" s="11" t="str">
+        <x:v>QA78</x:v>
+      </x:c>
+      <x:c r="B83" s="11" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C83" s="11" t="str">
+        <x:v>Permission après sortie</x:v>
+      </x:c>
+      <x:c r="D83" s="11" t="str">
+        <x:v>Différer getUserMedia, détruire la radio / quitter puis résoudre la permission.</x:v>
+      </x:c>
+      <x:c r="E83" s="11" t="str">
+        <x:v>Le résultat obsolète est fermé et ne ressuscite pas la session retirée.</x:v>
+      </x:c>
+      <x:c r="F83" s="13" t="str">
+        <x:v>Réussi</x:v>
+      </x:c>
+      <x:c r="G83" s="11" t="str">
+        <x:v>Test radio à promesse différée</x:v>
+      </x:c>
+      <x:c r="H83" s="11" t="str">
+        <x:v>Test réussi : un flux retourné après destruction de la radio est stoppé et la session reste inactive. Cette protection existante passait déjà avant le correctif et reste conservée. Aucun périphérique physique utilisé.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84" ht="64" customHeight="1">
+      <x:c r="A84" s="12" t="str">
+        <x:v>QA79</x:v>
+      </x:c>
+      <x:c r="B84" s="12" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C84" s="12" t="str">
+        <x:v>Réactivation concurrente</x:v>
+      </x:c>
+      <x:c r="D84" s="12" t="str">
+        <x:v>Désactiver, relancer puis résoudre/refuser l’ancienne demande ou son activation d’écoute dans différents ordres.</x:v>
+      </x:c>
+      <x:c r="E84" s="12" t="str">
+        <x:v>Flux récent, demande courante et écoute préservés ; ancien succès arrêté, ancien refus ou finaliseur sans effet sur l’état récent.</x:v>
+      </x:c>
+      <x:c r="F84" s="13" t="str">
+        <x:v>Réussi</x:v>
+      </x:c>
+      <x:c r="G84" s="12" t="str">
+        <x:v>Quatre tests radio de réactivation</x:v>
+      </x:c>
+      <x:c r="H84" s="12" t="str">
+        <x:v>Quatre tests réussis : ancien accord, ancien refus, ancienne finalisation et ancien échec d’écoute ne remplacent ni ne coupent le flux / la demande / l’écoute récents. Nouvel état PTT préservé et demande courante non dupliquée. API simulées.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85" ht="77" customHeight="1">
+      <x:c r="A85" s="11" t="str">
+        <x:v>QA80</x:v>
+      </x:c>
+      <x:c r="B85" s="11" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C85" s="11" t="str">
+        <x:v>Attente de l’interface</x:v>
+      </x:c>
+      <x:c r="D85" s="11" t="str">
+        <x:v>Lancer une permission différée, éteindre, réactiver puis terminer l’ancienne opération.</x:v>
+      </x:c>
+      <x:c r="E85" s="11" t="str">
+        <x:v>Nouvelle activation disponible ; les résultats anciens ne modifient pas l’état d’attente de l’opération récente.</x:v>
+      </x:c>
+      <x:c r="F85" s="13" t="str">
+        <x:v>Réussi</x:v>
+      </x:c>
+      <x:c r="G85" s="11" t="str">
+        <x:v>Tests du contrôleur UI</x:v>
+      </x:c>
+      <x:c r="H85" s="11" t="str">
+        <x:v>4/4 tests de radio-actions : arrêt libère l’attente ; ancienne réponse ignorée, refus courant signalé ; changement de salon / démontage invalide les callbacks ; appel dans le geste utilisateur et échec synchrone nettoyé. Typecheck réussi. Aucun test DOM, micro physique ou GPU.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86" ht="77" customHeight="1">
+      <x:c r="A86" s="12" t="str">
+        <x:v>QA81</x:v>
+      </x:c>
+      <x:c r="B86" s="12" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C86" s="12" t="str">
+        <x:v>Builds et édition portable</x:v>
+      </x:c>
+      <x:c r="D86" s="12" t="str">
+        <x:v>Compiler les éditions locale et hébergée ; lancer le serveur portable compilé avec deux clients HTTP, sans node_modules.</x:v>
+      </x:c>
+      <x:c r="E86" s="12" t="str">
+        <x:v>HTML servi ; modules serveur privés ; références et consensus justes ; départ des deux membres.</x:v>
+      </x:c>
+      <x:c r="F86" s="13" t="str">
+        <x:v>Réussi</x:v>
+      </x:c>
+      <x:c r="G86" s="12" t="str">
+        <x:v>Build / HTTP portable</x:v>
+      </x:c>
+      <x:c r="H86" s="12" t="str">
+        <x:v>v0.2.1 : typecheck, build local, build hébergé et test portable réussis. Deux clients HTTP authentifiés : référence, inspection, perceptions privées, unanimité et sortie ; serveur compilé lancé sans node_modules. Les archives finales et GitHub CI restent à contrôler après assemblage / publication.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="F6:F81">
+  <x:conditionalFormatting sqref="F6:F86">
     <x:cfRule type="containsText" dxfId="36" priority="1" operator="containsText" text="Bloqué"/>
     <x:cfRule type="containsText" dxfId="37" priority="2" operator="containsText" text="Validé"/>
     <x:cfRule type="containsText" dxfId="38" priority="3" operator="containsText" text="Réussi"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="F6:F81">
+    <x:dataValidation type="list" sqref="F6:F86">
       <x:formula1>"Présent,Prévu,Implémenté — QA partielle,Validé,À vérifier,Conçu — non implémenté,Bloqué,Réussi,Partiel,À exécuter,À tester sur GPU,À tester sur appareils,Conception définie,Contrôle structurel partiel"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re43065e9d1fd43cd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5e62a490fb44b8a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7065,7 +7247,7 @@
         <x:v>Source de vérité code</x:v>
       </x:c>
       <x:c r="C9" s="11" t="str">
-        <x:v>Catalogue runtime v0.2</x:v>
+        <x:v>Catalogue runtime 0.2.1</x:v>
       </x:c>
       <x:c r="D9" s="11" t="str">
         <x:v>54 identifiants intégrés ; titres, baseline, intensité, difficulté et lieux proviennent du code.</x:v>
@@ -7088,7 +7270,7 @@
         <x:v>Règles actuelles</x:v>
       </x:c>
       <x:c r="C10" s="12" t="str">
-        <x:v>Machine de jeu v0.2</x:v>
+        <x:v>Machine de jeu 0.2.1</x:v>
       </x:c>
       <x:c r="D10" s="12" t="str">
         <x:v>Campagne 3 × 3 avec paliers ; lieu unique 9 consécutifs ; 68 % d’anomalies ; 3 erreurs standard.</x:v>
@@ -7471,7 +7653,7 @@
         <x:v>Le panneau métro et le moniteur clinique sont des références fixes de jeu.</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="64" customHeight="1">
+    <x:row r="27" ht="77" customHeight="1">
       <x:c r="A27" s="11" t="str">
         <x:v>R22</x:v>
       </x:c>
@@ -7482,7 +7664,7 @@
         <x:v>Bilan de vérification</x:v>
       </x:c>
       <x:c r="D27" s="11" t="str">
-        <x:v>17 tests de règles, 12 tests radio, 11 suites géométriques CPU ; D1 local quatre clients et neuf tours réussi. Deux onglets : offre/réponse échangées, mais zéro candidat ICE et aucun audio connecté. GLB relu avec trois clips.</x:v>
+        <x:v>v0.2.1 : 19 tests radio et 4 du contrôleur UI réussis ; typecheck, builds local / hébergé et test portable à deux clients HTTP réussis. Preuves v0.2 conservées : 17 règles, 11 suites CPU 3D, D1 quatre clients et GLB relu. Aucun nouvel essai ICE ou de microphone physique.</x:v>
       </x:c>
       <x:c r="E27" s="11" t="str">
         <x:v>docs/QA.md</x:v>
@@ -7586,10 +7768,79 @@
         <x:v>Modèle procédural original ; pas de skinning, pas de lettrage badge embarqué et pas de validation GPU.</x:v>
       </x:c>
     </x:row>
+    <x:row r="32" ht="64" customHeight="1">
+      <x:c r="A32" s="12" t="str">
+        <x:v>R27</x:v>
+      </x:c>
+      <x:c r="B32" s="12" t="str">
+        <x:v>Correctif vérifié</x:v>
+      </x:c>
+      <x:c r="C32" s="12" t="str">
+        <x:v>Autorisation micro tardive · 0.2.1</x:v>
+      </x:c>
+      <x:c r="D32" s="12" t="str">
+        <x:v>Invalider les demandes obsolètes, arrêter leurs flux retournés et préserver la réactivation la plus récente.</x:v>
+      </x:c>
+      <x:c r="E32" s="12" t="str">
+        <x:v>docs/qa-radio-cancellation-v0.2.1.json ; tests/radio.test.mjs</x:v>
+      </x:c>
+      <x:c r="F32" s="20" t="d">
+        <x:v>2026-10-26T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="G32" s="12" t="str">
+        <x:v>19/19 tests radio réussis, dont 7 nouveaux : extinction, micro seul, anciennes réponses, nouvelle demande et sortie. Avant correction : 6 échecs / 1 succès ; après : 7/7. Pistes et API simulées ; aucun microphone physique ni transmission mesurée.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="77" customHeight="1">
+      <x:c r="A33" s="11" t="str">
+        <x:v>R28</x:v>
+      </x:c>
+      <x:c r="B33" s="11" t="str">
+        <x:v>Contrôleur vérifié</x:v>
+      </x:c>
+      <x:c r="C33" s="11" t="str">
+        <x:v>État d’attente de la radio · 0.2.1</x:v>
+      </x:c>
+      <x:c r="D33" s="11" t="str">
+        <x:v>Annuler l’opération UI retirée afin qu’une permission encore ouverte ne bloque pas la commande suivante.</x:v>
+      </x:c>
+      <x:c r="E33" s="11" t="str">
+        <x:v>docs/qa-radio-ui-v0.2.1.json ; tests/radio-actions.test.mjs</x:v>
+      </x:c>
+      <x:c r="F33" s="22" t="d">
+        <x:v>2026-10-26T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="G33" s="11" t="str">
+        <x:v>4/4 tests de radio-actions : arrêt libère l’attente ; ancienne réponse ignorée, refus courant signalé ; changement de salon / démontage invalide les callbacks ; appel dans le geste utilisateur et échec synchrone nettoyé. Typecheck réussi. Aucun test DOM, micro physique ou GPU.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="77" customHeight="1">
+      <x:c r="A34" s="12" t="str">
+        <x:v>R29</x:v>
+      </x:c>
+      <x:c r="B34" s="12" t="str">
+        <x:v>Livraison vérifiée</x:v>
+      </x:c>
+      <x:c r="C34" s="12" t="str">
+        <x:v>Compilation et serveur portable · 0.2.1</x:v>
+      </x:c>
+      <x:c r="D34" s="12" t="str">
+        <x:v>Typecheck, builds local / hébergé et parcours HTTP portable à deux clients exécutés.</x:v>
+      </x:c>
+      <x:c r="E34" s="12" t="str">
+        <x:v>docs/qa-final-v0.2.1.json ; .github/workflows/ci.yml</x:v>
+      </x:c>
+      <x:c r="F34" s="20" t="d">
+        <x:v>2026-10-26T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="G34" s="12" t="str">
+        <x:v>v0.2.1 : typecheck, build local, build hébergé et test portable réussis. Deux clients HTTP authentifiés : référence, inspection, perceptions privées, unanimité et sortie ; serveur compilé lancé sans node_modules. Les archives finales et GitHub CI restent à contrôler après assemblage / publication.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43fd63bcae4a42e5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f1c5233b67e42d4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8304,7 +8555,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref7778cb633344f1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55c3b554c7314ae1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8508,7 +8759,7 @@
         <x:v>Canal de preuve</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="64" customHeight="1">
+    <x:row r="6" ht="77" customHeight="1">
       <x:c r="A6" s="12" t="str">
         <x:v>PX-001</x:v>
       </x:c>
@@ -8561,7 +8812,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R6" s="12" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S6" s="18" t="str">
         <x:v>Oui</x:v>
@@ -8576,7 +8827,7 @@
         <x:v>Visuel / objet / espace</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="64" customHeight="1">
+    <x:row r="7" ht="77" customHeight="1">
       <x:c r="A7" s="11" t="str">
         <x:v>PX-002</x:v>
       </x:c>
@@ -8629,7 +8880,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="R7" s="11" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S7" s="19" t="str">
         <x:v>Oui</x:v>
@@ -8644,7 +8895,7 @@
         <x:v>Visuel / objet / espace</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="64" customHeight="1">
+    <x:row r="8" ht="77" customHeight="1">
       <x:c r="A8" s="12" t="str">
         <x:v>PX-003</x:v>
       </x:c>
@@ -8697,7 +8948,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R8" s="12" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S8" s="18" t="str">
         <x:v>Oui</x:v>
@@ -8712,7 +8963,7 @@
         <x:v>Visuel / objet / espace</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="64" customHeight="1">
+    <x:row r="9" ht="77" customHeight="1">
       <x:c r="A9" s="11" t="str">
         <x:v>PX-004</x:v>
       </x:c>
@@ -8765,7 +9016,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R9" s="11" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S9" s="19" t="str">
         <x:v>Oui</x:v>
@@ -8780,7 +9031,7 @@
         <x:v>Visuel / objet / espace</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="64" customHeight="1">
+    <x:row r="10" ht="77" customHeight="1">
       <x:c r="A10" s="12" t="str">
         <x:v>PX-005</x:v>
       </x:c>
@@ -8833,7 +9084,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R10" s="12" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S10" s="18" t="str">
         <x:v>Oui</x:v>
@@ -8848,7 +9099,7 @@
         <x:v>Visuel / objet / espace</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="64" customHeight="1">
+    <x:row r="11" ht="77" customHeight="1">
       <x:c r="A11" s="11" t="str">
         <x:v>PX-006</x:v>
       </x:c>
@@ -8901,7 +9152,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="R11" s="11" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S11" s="19" t="str">
         <x:v>Oui</x:v>
@@ -8916,7 +9167,7 @@
         <x:v>Visuel / objet / espace</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="64" customHeight="1">
+    <x:row r="12" ht="77" customHeight="1">
       <x:c r="A12" s="12" t="str">
         <x:v>PX-007</x:v>
       </x:c>
@@ -8969,7 +9220,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R12" s="12" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S12" s="18" t="str">
         <x:v>Oui</x:v>
@@ -8984,7 +9235,7 @@
         <x:v>Visuel / objet / espace</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="64" customHeight="1">
+    <x:row r="13" ht="77" customHeight="1">
       <x:c r="A13" s="11" t="str">
         <x:v>PX-008</x:v>
       </x:c>
@@ -9037,7 +9288,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="R13" s="11" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S13" s="19" t="str">
         <x:v>Oui</x:v>
@@ -9052,7 +9303,7 @@
         <x:v>Visuel / objet / espace</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="64" customHeight="1">
+    <x:row r="14" ht="77" customHeight="1">
       <x:c r="A14" s="12" t="str">
         <x:v>PX-009</x:v>
       </x:c>
@@ -9105,7 +9356,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R14" s="12" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S14" s="18" t="str">
         <x:v>Oui</x:v>
@@ -9120,7 +9371,7 @@
         <x:v>Visuel / objet / espace</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="64" customHeight="1">
+    <x:row r="15" ht="77" customHeight="1">
       <x:c r="A15" s="11" t="str">
         <x:v>PX-010</x:v>
       </x:c>
@@ -9173,7 +9424,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="R15" s="11" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S15" s="19" t="str">
         <x:v>Oui</x:v>
@@ -9188,7 +9439,7 @@
         <x:v>Visuel / objet / espace</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="64" customHeight="1">
+    <x:row r="16" ht="77" customHeight="1">
       <x:c r="A16" s="12" t="str">
         <x:v>PX-011</x:v>
       </x:c>
@@ -9241,7 +9492,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="R16" s="12" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S16" s="18" t="str">
         <x:v>Oui</x:v>
@@ -9256,7 +9507,7 @@
         <x:v>Visuel / objet / espace</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="64" customHeight="1">
+    <x:row r="17" ht="77" customHeight="1">
       <x:c r="A17" s="11" t="str">
         <x:v>PX-012</x:v>
       </x:c>
@@ -9309,7 +9560,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="R17" s="11" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S17" s="19" t="str">
         <x:v>Oui</x:v>
@@ -9324,7 +9575,7 @@
         <x:v>Visuel / objet / espace</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="64" customHeight="1">
+    <x:row r="18" ht="77" customHeight="1">
       <x:c r="A18" s="12" t="str">
         <x:v>PX-013</x:v>
       </x:c>
@@ -9377,7 +9628,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R18" s="12" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S18" s="18" t="str">
         <x:v>Oui</x:v>
@@ -9392,7 +9643,7 @@
         <x:v>Visuel / objet / espace</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="64" customHeight="1">
+    <x:row r="19" ht="77" customHeight="1">
       <x:c r="A19" s="11" t="str">
         <x:v>PX-014</x:v>
       </x:c>
@@ -9445,7 +9696,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R19" s="11" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S19" s="19" t="str">
         <x:v>Oui</x:v>
@@ -9460,7 +9711,7 @@
         <x:v>Visuel / objet / espace</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="64" customHeight="1">
+    <x:row r="20" ht="77" customHeight="1">
       <x:c r="A20" s="12" t="str">
         <x:v>PX-015</x:v>
       </x:c>
@@ -9513,7 +9764,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R20" s="12" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S20" s="18" t="str">
         <x:v>Oui</x:v>
@@ -9528,7 +9779,7 @@
         <x:v>Visuel / objet / espace</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="64" customHeight="1">
+    <x:row r="21" ht="77" customHeight="1">
       <x:c r="A21" s="11" t="str">
         <x:v>PX-016</x:v>
       </x:c>
@@ -9581,7 +9832,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="R21" s="11" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S21" s="19" t="str">
         <x:v>Oui</x:v>
@@ -9596,7 +9847,7 @@
         <x:v>Visuel / objet / espace</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="64" customHeight="1">
+    <x:row r="22" ht="77" customHeight="1">
       <x:c r="A22" s="12" t="str">
         <x:v>PX-017</x:v>
       </x:c>
@@ -9649,7 +9900,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R22" s="12" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S22" s="18" t="str">
         <x:v>Oui</x:v>
@@ -9664,7 +9915,7 @@
         <x:v>Visuel / objet / espace</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="64" customHeight="1">
+    <x:row r="23" ht="77" customHeight="1">
       <x:c r="A23" s="11" t="str">
         <x:v>PX-018</x:v>
       </x:c>
@@ -9717,7 +9968,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="R23" s="11" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S23" s="19" t="str">
         <x:v>Oui</x:v>
@@ -9732,7 +9983,7 @@
         <x:v>Visuel / objet / espace</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="64" customHeight="1">
+    <x:row r="24" ht="77" customHeight="1">
       <x:c r="A24" s="12" t="str">
         <x:v>PX-019</x:v>
       </x:c>
@@ -9785,7 +10036,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R24" s="12" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S24" s="18" t="str">
         <x:v>Oui</x:v>
@@ -9800,7 +10051,7 @@
         <x:v>Visuel / objet / espace</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" ht="64" customHeight="1">
+    <x:row r="25" ht="77" customHeight="1">
       <x:c r="A25" s="11" t="str">
         <x:v>PX-020</x:v>
       </x:c>
@@ -9853,7 +10104,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="R25" s="11" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S25" s="19" t="str">
         <x:v>Oui</x:v>
@@ -9868,7 +10119,7 @@
         <x:v>Visuel / objet / espace</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="64" customHeight="1">
+    <x:row r="26" ht="77" customHeight="1">
       <x:c r="A26" s="12" t="str">
         <x:v>PX-021</x:v>
       </x:c>
@@ -9921,7 +10172,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="R26" s="12" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S26" s="18" t="str">
         <x:v>Oui</x:v>
@@ -9936,7 +10187,7 @@
         <x:v>Visuel / objet / espace</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="64" customHeight="1">
+    <x:row r="27" ht="77" customHeight="1">
       <x:c r="A27" s="11" t="str">
         <x:v>PX-022</x:v>
       </x:c>
@@ -9989,7 +10240,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R27" s="11" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S27" s="19" t="str">
         <x:v>Oui</x:v>
@@ -10004,7 +10255,7 @@
         <x:v>Visuel / objet / espace</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" ht="64" customHeight="1">
+    <x:row r="28" ht="77" customHeight="1">
       <x:c r="A28" s="12" t="str">
         <x:v>PX-023</x:v>
       </x:c>
@@ -10057,7 +10308,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R28" s="12" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S28" s="18" t="str">
         <x:v>Oui</x:v>
@@ -10072,7 +10323,7 @@
         <x:v>Visuel / objet / espace</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="64" customHeight="1">
+    <x:row r="29" ht="77" customHeight="1">
       <x:c r="A29" s="11" t="str">
         <x:v>PX-024</x:v>
       </x:c>
@@ -10125,7 +10376,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R29" s="11" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S29" s="19" t="str">
         <x:v>Oui</x:v>
@@ -10140,7 +10391,7 @@
         <x:v>Corps / reflet / mouvement</x:v>
       </x:c>
     </x:row>
-    <x:row r="30" ht="64" customHeight="1">
+    <x:row r="30" ht="77" customHeight="1">
       <x:c r="A30" s="12" t="str">
         <x:v>PX-025</x:v>
       </x:c>
@@ -10193,7 +10444,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="R30" s="12" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S30" s="18" t="str">
         <x:v>Oui</x:v>
@@ -10261,7 +10512,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="R31" s="11" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S31" s="19" t="str">
         <x:v>—</x:v>
@@ -10276,7 +10527,7 @@
         <x:v>Comparaison entre témoins</x:v>
       </x:c>
     </x:row>
-    <x:row r="32" ht="64" customHeight="1">
+    <x:row r="32" ht="77" customHeight="1">
       <x:c r="A32" s="12" t="str">
         <x:v>PX-027</x:v>
       </x:c>
@@ -10329,7 +10580,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="R32" s="12" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S32" s="18" t="str">
         <x:v>Oui</x:v>
@@ -10397,7 +10648,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="R33" s="11" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S33" s="19" t="str">
         <x:v>—</x:v>
@@ -10465,7 +10716,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="R34" s="12" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S34" s="18" t="str">
         <x:v>—</x:v>
@@ -10533,7 +10784,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="R35" s="11" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S35" s="19" t="str">
         <x:v>—</x:v>
@@ -10601,7 +10852,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="R36" s="12" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S36" s="18" t="str">
         <x:v>—</x:v>
@@ -10616,7 +10867,7 @@
         <x:v>Comparaison entre témoins</x:v>
       </x:c>
     </x:row>
-    <x:row r="37" ht="64" customHeight="1">
+    <x:row r="37" ht="77" customHeight="1">
       <x:c r="A37" s="11" t="str">
         <x:v>PX-032</x:v>
       </x:c>
@@ -10669,7 +10920,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="R37" s="11" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S37" s="19" t="str">
         <x:v>Oui</x:v>
@@ -10737,7 +10988,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R38" s="12" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S38" s="18" t="str">
         <x:v>—</x:v>
@@ -10805,7 +11056,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="R39" s="11" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S39" s="19" t="str">
         <x:v>—</x:v>
@@ -10873,7 +11124,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="R40" s="12" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S40" s="18" t="str">
         <x:v>—</x:v>
@@ -10941,7 +11192,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="R41" s="11" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S41" s="19" t="str">
         <x:v>—</x:v>
@@ -11009,7 +11260,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R42" s="12" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S42" s="18" t="str">
         <x:v>—</x:v>
@@ -11077,7 +11328,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R43" s="11" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S43" s="19" t="str">
         <x:v>—</x:v>
@@ -11145,7 +11396,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R44" s="12" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S44" s="18" t="str">
         <x:v>—</x:v>
@@ -11213,7 +11464,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R45" s="11" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S45" s="19" t="str">
         <x:v>—</x:v>
@@ -11281,7 +11532,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R46" s="12" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S46" s="18" t="str">
         <x:v>—</x:v>
@@ -11349,7 +11600,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R47" s="11" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S47" s="19" t="str">
         <x:v>—</x:v>
@@ -11417,7 +11668,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R48" s="12" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S48" s="18" t="str">
         <x:v>—</x:v>
@@ -11485,7 +11736,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R49" s="11" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S49" s="19" t="str">
         <x:v>—</x:v>
@@ -11553,7 +11804,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R50" s="12" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S50" s="18" t="str">
         <x:v>—</x:v>
@@ -11621,7 +11872,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R51" s="11" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S51" s="19" t="str">
         <x:v>—</x:v>
@@ -11689,7 +11940,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R52" s="12" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S52" s="18" t="str">
         <x:v>—</x:v>
@@ -11757,7 +12008,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R53" s="11" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S53" s="19" t="str">
         <x:v>—</x:v>
@@ -11825,7 +12076,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R54" s="12" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S54" s="18" t="str">
         <x:v>—</x:v>
@@ -11893,7 +12144,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R55" s="11" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S55" s="19" t="str">
         <x:v>—</x:v>
@@ -11908,7 +12159,7 @@
         <x:v>Visuel / objet / espace</x:v>
       </x:c>
     </x:row>
-    <x:row r="56" ht="64" customHeight="1">
+    <x:row r="56" ht="77" customHeight="1">
       <x:c r="A56" s="12" t="str">
         <x:v>PX-051</x:v>
       </x:c>
@@ -11961,7 +12212,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R56" s="12" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S56" s="18" t="str">
         <x:v>—</x:v>
@@ -11976,7 +12227,7 @@
         <x:v>Visuel / objet / espace</x:v>
       </x:c>
     </x:row>
-    <x:row r="57" ht="64" customHeight="1">
+    <x:row r="57" ht="77" customHeight="1">
       <x:c r="A57" s="11" t="str">
         <x:v>PX-052</x:v>
       </x:c>
@@ -12029,7 +12280,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R57" s="11" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S57" s="19" t="str">
         <x:v>Oui</x:v>
@@ -12097,7 +12348,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R58" s="12" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S58" s="18" t="str">
         <x:v>—</x:v>
@@ -12165,7 +12416,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R59" s="11" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S59" s="19" t="str">
         <x:v>—</x:v>
@@ -12233,7 +12484,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R60" s="12" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S60" s="18" t="str">
         <x:v>—</x:v>
@@ -12248,7 +12499,7 @@
         <x:v>Visuel / objet / espace</x:v>
       </x:c>
     </x:row>
-    <x:row r="61" ht="64" customHeight="1">
+    <x:row r="61" ht="77" customHeight="1">
       <x:c r="A61" s="11" t="str">
         <x:v>PX-056</x:v>
       </x:c>
@@ -12301,7 +12552,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R61" s="11" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S61" s="19" t="str">
         <x:v>Oui</x:v>
@@ -12369,7 +12620,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R62" s="12" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S62" s="18" t="str">
         <x:v>—</x:v>
@@ -12437,7 +12688,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R63" s="11" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S63" s="19" t="str">
         <x:v>—</x:v>
@@ -12505,7 +12756,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R64" s="12" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S64" s="18" t="str">
         <x:v>—</x:v>
@@ -12520,7 +12771,7 @@
         <x:v>Visuel / objet / espace</x:v>
       </x:c>
     </x:row>
-    <x:row r="65" ht="64" customHeight="1">
+    <x:row r="65" ht="77" customHeight="1">
       <x:c r="A65" s="11" t="str">
         <x:v>PX-060</x:v>
       </x:c>
@@ -12573,7 +12824,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R65" s="11" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S65" s="19" t="str">
         <x:v>Oui</x:v>
@@ -12641,7 +12892,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R66" s="12" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S66" s="18" t="str">
         <x:v>—</x:v>
@@ -12709,7 +12960,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R67" s="11" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S67" s="19" t="str">
         <x:v>—</x:v>
@@ -12777,7 +13028,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R68" s="12" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S68" s="18" t="str">
         <x:v>—</x:v>
@@ -12845,7 +13096,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R69" s="11" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S69" s="19" t="str">
         <x:v>—</x:v>
@@ -12913,7 +13164,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R70" s="12" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S70" s="18" t="str">
         <x:v>—</x:v>
@@ -12928,7 +13179,7 @@
         <x:v>Visuel / objet / espace</x:v>
       </x:c>
     </x:row>
-    <x:row r="71" ht="64" customHeight="1">
+    <x:row r="71" ht="77" customHeight="1">
       <x:c r="A71" s="11" t="str">
         <x:v>PX-066</x:v>
       </x:c>
@@ -12981,7 +13232,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R71" s="11" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S71" s="19" t="str">
         <x:v>Oui</x:v>
@@ -13049,7 +13300,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R72" s="12" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S72" s="18" t="str">
         <x:v>—</x:v>
@@ -13117,7 +13368,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R73" s="11" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S73" s="19" t="str">
         <x:v>—</x:v>
@@ -13185,7 +13436,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R74" s="12" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S74" s="18" t="str">
         <x:v>—</x:v>
@@ -13253,7 +13504,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R75" s="11" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S75" s="19" t="str">
         <x:v>—</x:v>
@@ -13321,7 +13572,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R76" s="12" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S76" s="18" t="str">
         <x:v>—</x:v>
@@ -13389,7 +13640,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="R77" s="11" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S77" s="19" t="str">
         <x:v>—</x:v>
@@ -13457,7 +13708,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R78" s="12" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S78" s="18" t="str">
         <x:v>—</x:v>
@@ -13525,7 +13776,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R79" s="11" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S79" s="19" t="str">
         <x:v>—</x:v>
@@ -13593,7 +13844,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R80" s="12" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S80" s="18" t="str">
         <x:v>—</x:v>
@@ -13661,7 +13912,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R81" s="11" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S81" s="19" t="str">
         <x:v>—</x:v>
@@ -13729,7 +13980,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R82" s="12" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S82" s="18" t="str">
         <x:v>—</x:v>
@@ -13744,7 +13995,7 @@
         <x:v>Visuel / objet / espace</x:v>
       </x:c>
     </x:row>
-    <x:row r="83" ht="64" customHeight="1">
+    <x:row r="83" ht="77" customHeight="1">
       <x:c r="A83" s="11" t="str">
         <x:v>PX-078</x:v>
       </x:c>
@@ -13797,7 +14048,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R83" s="11" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S83" s="19" t="str">
         <x:v>—</x:v>
@@ -13812,7 +14063,7 @@
         <x:v>Visuel / objet / espace</x:v>
       </x:c>
     </x:row>
-    <x:row r="84" ht="64" customHeight="1">
+    <x:row r="84" ht="77" customHeight="1">
       <x:c r="A84" s="12" t="str">
         <x:v>PX-079</x:v>
       </x:c>
@@ -13865,7 +14116,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R84" s="12" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S84" s="18" t="str">
         <x:v>—</x:v>
@@ -13933,7 +14184,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R85" s="11" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S85" s="19" t="str">
         <x:v>—</x:v>
@@ -13948,7 +14199,7 @@
         <x:v>Visuel / objet / espace</x:v>
       </x:c>
     </x:row>
-    <x:row r="86" ht="64" customHeight="1">
+    <x:row r="86" ht="77" customHeight="1">
       <x:c r="A86" s="12" t="str">
         <x:v>PX-081</x:v>
       </x:c>
@@ -14001,7 +14252,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R86" s="12" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S86" s="18" t="str">
         <x:v>Oui</x:v>
@@ -14016,7 +14267,7 @@
         <x:v>Corps / reflet / mouvement</x:v>
       </x:c>
     </x:row>
-    <x:row r="87" ht="64" customHeight="1">
+    <x:row r="87" ht="77" customHeight="1">
       <x:c r="A87" s="11" t="str">
         <x:v>PX-082</x:v>
       </x:c>
@@ -14069,7 +14320,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R87" s="11" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S87" s="19" t="str">
         <x:v>Oui</x:v>
@@ -14084,7 +14335,7 @@
         <x:v>Corps / reflet / mouvement</x:v>
       </x:c>
     </x:row>
-    <x:row r="88" ht="64" customHeight="1">
+    <x:row r="88" ht="77" customHeight="1">
       <x:c r="A88" s="12" t="str">
         <x:v>PX-083</x:v>
       </x:c>
@@ -14137,7 +14388,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R88" s="12" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S88" s="18" t="str">
         <x:v>Oui</x:v>
@@ -14152,7 +14403,7 @@
         <x:v>Corps / reflet / mouvement</x:v>
       </x:c>
     </x:row>
-    <x:row r="89" ht="64" customHeight="1">
+    <x:row r="89" ht="77" customHeight="1">
       <x:c r="A89" s="11" t="str">
         <x:v>PX-084</x:v>
       </x:c>
@@ -14205,7 +14456,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R89" s="11" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S89" s="19" t="str">
         <x:v>Oui</x:v>
@@ -14220,7 +14471,7 @@
         <x:v>Corps / reflet / mouvement</x:v>
       </x:c>
     </x:row>
-    <x:row r="90" ht="64" customHeight="1">
+    <x:row r="90" ht="77" customHeight="1">
       <x:c r="A90" s="12" t="str">
         <x:v>PX-085</x:v>
       </x:c>
@@ -14273,7 +14524,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R90" s="12" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S90" s="18" t="str">
         <x:v>Oui</x:v>
@@ -14288,7 +14539,7 @@
         <x:v>Corps / reflet / mouvement</x:v>
       </x:c>
     </x:row>
-    <x:row r="91" ht="64" customHeight="1">
+    <x:row r="91" ht="77" customHeight="1">
       <x:c r="A91" s="11" t="str">
         <x:v>PX-086</x:v>
       </x:c>
@@ -14341,7 +14592,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="R91" s="11" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S91" s="19" t="str">
         <x:v>Oui</x:v>
@@ -14356,7 +14607,7 @@
         <x:v>Visuel / objet / espace</x:v>
       </x:c>
     </x:row>
-    <x:row r="92" ht="64" customHeight="1">
+    <x:row r="92" ht="77" customHeight="1">
       <x:c r="A92" s="12" t="str">
         <x:v>PX-087</x:v>
       </x:c>
@@ -14409,7 +14660,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="R92" s="12" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S92" s="18" t="str">
         <x:v>—</x:v>
@@ -14424,7 +14675,7 @@
         <x:v>Visuel / objet / espace</x:v>
       </x:c>
     </x:row>
-    <x:row r="93" ht="64" customHeight="1">
+    <x:row r="93" ht="77" customHeight="1">
       <x:c r="A93" s="11" t="str">
         <x:v>PX-088</x:v>
       </x:c>
@@ -14477,7 +14728,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R93" s="11" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S93" s="19" t="str">
         <x:v>—</x:v>
@@ -14492,7 +14743,7 @@
         <x:v>Visuel / objet / espace</x:v>
       </x:c>
     </x:row>
-    <x:row r="94" ht="64" customHeight="1">
+    <x:row r="94" ht="77" customHeight="1">
       <x:c r="A94" s="12" t="str">
         <x:v>PX-089</x:v>
       </x:c>
@@ -14545,7 +14796,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R94" s="12" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S94" s="18" t="str">
         <x:v>—</x:v>
@@ -14560,7 +14811,7 @@
         <x:v>Visuel / objet / espace</x:v>
       </x:c>
     </x:row>
-    <x:row r="95" ht="64" customHeight="1">
+    <x:row r="95" ht="77" customHeight="1">
       <x:c r="A95" s="11" t="str">
         <x:v>PX-090</x:v>
       </x:c>
@@ -14613,7 +14864,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R95" s="11" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S95" s="19" t="str">
         <x:v>—</x:v>
@@ -14628,7 +14879,7 @@
         <x:v>Visuel / objet / espace</x:v>
       </x:c>
     </x:row>
-    <x:row r="96" ht="64" customHeight="1">
+    <x:row r="96" ht="77" customHeight="1">
       <x:c r="A96" s="12" t="str">
         <x:v>PX-091</x:v>
       </x:c>
@@ -14681,7 +14932,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="R96" s="12" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S96" s="18" t="str">
         <x:v>—</x:v>
@@ -14696,7 +14947,7 @@
         <x:v>Visuel / objet / espace</x:v>
       </x:c>
     </x:row>
-    <x:row r="97" ht="64" customHeight="1">
+    <x:row r="97" ht="77" customHeight="1">
       <x:c r="A97" s="11" t="str">
         <x:v>PX-092</x:v>
       </x:c>
@@ -14749,7 +15000,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R97" s="11" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S97" s="19" t="str">
         <x:v>—</x:v>
@@ -14764,7 +15015,7 @@
         <x:v>Visuel / objet / espace</x:v>
       </x:c>
     </x:row>
-    <x:row r="98" ht="64" customHeight="1">
+    <x:row r="98" ht="77" customHeight="1">
       <x:c r="A98" s="12" t="str">
         <x:v>PX-093</x:v>
       </x:c>
@@ -14817,7 +15068,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R98" s="12" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S98" s="18" t="str">
         <x:v>—</x:v>
@@ -14832,7 +15083,7 @@
         <x:v>Visuel / objet / espace</x:v>
       </x:c>
     </x:row>
-    <x:row r="99" ht="64" customHeight="1">
+    <x:row r="99" ht="77" customHeight="1">
       <x:c r="A99" s="11" t="str">
         <x:v>PX-094</x:v>
       </x:c>
@@ -14885,7 +15136,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R99" s="11" t="str">
-        <x:v>ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
+        <x:v>Preuves v0.2 conservées : ID intégré au catalogue et aux règles. 17 tests de règles couvrent les 54 cas ; 11 suites CPU couvrent 48 preuves visuelles et leur reset. Pixels, shaders, reflet final et FPS restent à tester sur GPU réel.</x:v>
       </x:c>
       <x:c r="S99" s="19" t="str">
         <x:v>—</x:v>
@@ -14953,7 +15204,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R100" s="12" t="str">
-        <x:v>Réception WebAudio et calibration déterministe intégrées. 12 tests radio réussis, dont relevés sans micro/réseau, PTT et consentement. Écoute humaine, microphones physiques et TURN réel restent à éprouver.</x:v>
+        <x:v>Réception WebAudio et calibration déterministe intégrées. 19 tests radio réussis, dont relevés sans micro/réseau, PTT, consentement et annulation des demandes micro obsolètes. Écoute humaine, microphones physiques et TURN réel restent à éprouver.</x:v>
       </x:c>
       <x:c r="S100" s="18" t="str">
         <x:v>Oui</x:v>
@@ -15021,7 +15272,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R101" s="11" t="str">
-        <x:v>Réception WebAudio et calibration déterministe intégrées. 12 tests radio réussis, dont relevés sans micro/réseau, PTT et consentement. Écoute humaine, microphones physiques et TURN réel restent à éprouver.</x:v>
+        <x:v>Réception WebAudio et calibration déterministe intégrées. 19 tests radio réussis, dont relevés sans micro/réseau, PTT, consentement et annulation des demandes micro obsolètes. Écoute humaine, microphones physiques et TURN réel restent à éprouver.</x:v>
       </x:c>
       <x:c r="S101" s="19" t="str">
         <x:v>Oui</x:v>
@@ -15089,7 +15340,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R102" s="12" t="str">
-        <x:v>Réception WebAudio et calibration déterministe intégrées. 12 tests radio réussis, dont relevés sans micro/réseau, PTT et consentement. Écoute humaine, microphones physiques et TURN réel restent à éprouver.</x:v>
+        <x:v>Réception WebAudio et calibration déterministe intégrées. 19 tests radio réussis, dont relevés sans micro/réseau, PTT, consentement et annulation des demandes micro obsolètes. Écoute humaine, microphones physiques et TURN réel restent à éprouver.</x:v>
       </x:c>
       <x:c r="S102" s="18" t="str">
         <x:v>Oui</x:v>
@@ -15157,7 +15408,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R103" s="11" t="str">
-        <x:v>Réception WebAudio et calibration déterministe intégrées. 12 tests radio réussis, dont relevés sans micro/réseau, PTT et consentement. Écoute humaine, microphones physiques et TURN réel restent à éprouver.</x:v>
+        <x:v>Réception WebAudio et calibration déterministe intégrées. 19 tests radio réussis, dont relevés sans micro/réseau, PTT, consentement et annulation des demandes micro obsolètes. Écoute humaine, microphones physiques et TURN réel restent à éprouver.</x:v>
       </x:c>
       <x:c r="S103" s="19" t="str">
         <x:v>Oui</x:v>
@@ -15225,7 +15476,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="R104" s="12" t="str">
-        <x:v>Réception WebAudio et calibration déterministe intégrées. 12 tests radio réussis, dont relevés sans micro/réseau, PTT et consentement. Écoute humaine, microphones physiques et TURN réel restent à éprouver.</x:v>
+        <x:v>Réception WebAudio et calibration déterministe intégrées. 19 tests radio réussis, dont relevés sans micro/réseau, PTT, consentement et annulation des demandes micro obsolètes. Écoute humaine, microphones physiques et TURN réel restent à éprouver.</x:v>
       </x:c>
       <x:c r="S104" s="18" t="str">
         <x:v>Oui</x:v>
@@ -15293,7 +15544,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R105" s="11" t="str">
-        <x:v>Réception WebAudio et calibration déterministe intégrées. 12 tests radio réussis, dont relevés sans micro/réseau, PTT et consentement. Écoute humaine, microphones physiques et TURN réel restent à éprouver.</x:v>
+        <x:v>Réception WebAudio et calibration déterministe intégrées. 19 tests radio réussis, dont relevés sans micro/réseau, PTT, consentement et annulation des demandes micro obsolètes. Écoute humaine, microphones physiques et TURN réel restent à éprouver.</x:v>
       </x:c>
       <x:c r="S105" s="19" t="str">
         <x:v>Oui</x:v>
@@ -15361,7 +15612,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R106" s="12" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S106" s="18" t="str">
         <x:v>—</x:v>
@@ -15429,7 +15680,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R107" s="11" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S107" s="19" t="str">
         <x:v>—</x:v>
@@ -15497,7 +15748,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R108" s="12" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S108" s="18" t="str">
         <x:v>—</x:v>
@@ -15565,7 +15816,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R109" s="11" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S109" s="19" t="str">
         <x:v>—</x:v>
@@ -15633,7 +15884,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R110" s="12" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S110" s="18" t="str">
         <x:v>—</x:v>
@@ -15701,7 +15952,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R111" s="11" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S111" s="19" t="str">
         <x:v>—</x:v>
@@ -15769,7 +16020,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R112" s="12" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S112" s="18" t="str">
         <x:v>—</x:v>
@@ -15837,7 +16088,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R113" s="11" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S113" s="19" t="str">
         <x:v>—</x:v>
@@ -15905,7 +16156,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R114" s="12" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S114" s="18" t="str">
         <x:v>—</x:v>
@@ -15973,7 +16224,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R115" s="11" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S115" s="19" t="str">
         <x:v>—</x:v>
@@ -16041,7 +16292,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R116" s="12" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S116" s="18" t="str">
         <x:v>—</x:v>
@@ -16109,7 +16360,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R117" s="11" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S117" s="19" t="str">
         <x:v>—</x:v>
@@ -16177,7 +16428,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R118" s="12" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S118" s="18" t="str">
         <x:v>—</x:v>
@@ -16245,7 +16496,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R119" s="11" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S119" s="19" t="str">
         <x:v>—</x:v>
@@ -16313,7 +16564,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R120" s="12" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S120" s="18" t="str">
         <x:v>—</x:v>
@@ -16381,7 +16632,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R121" s="11" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S121" s="19" t="str">
         <x:v>—</x:v>
@@ -16449,7 +16700,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R122" s="12" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S122" s="18" t="str">
         <x:v>—</x:v>
@@ -16517,7 +16768,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R123" s="11" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S123" s="19" t="str">
         <x:v>—</x:v>
@@ -16585,7 +16836,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R124" s="12" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S124" s="18" t="str">
         <x:v>—</x:v>
@@ -16653,7 +16904,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R125" s="11" t="str">
-        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.</x:v>
+        <x:v>Spécification originale ; effet absent du catalogue runtime v0.2.1.</x:v>
       </x:c>
       <x:c r="S125" s="19" t="str">
         <x:v>—</x:v>
@@ -16689,7 +16940,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbad04e8c4c964606"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c06891e25be4b15"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17000,7 +17251,7 @@
         <x:v>Rejouer une mutation après conflit seulement si elle reste valide.</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="64" customHeight="1">
+    <x:row r="16" ht="77" customHeight="1">
       <x:c r="A16" s="12" t="str">
         <x:v>C11</x:v>
       </x:c>
@@ -17017,7 +17268,7 @@
         <x:v>Implémenté — QA partielle</x:v>
       </x:c>
       <x:c r="F16" s="12" t="str">
-        <x:v>D1 local réel : quatre clients HTTP, neuf consensus concurrents, campagne trois lieux et références propres, signalisation privée et départ réussis. Ni microphones physiques ni trajet TURN réel testés par ce rapport.</x:v>
+        <x:v>Rapport v0.2 conservé : D1 local réel : quatre clients HTTP, neuf consensus concurrents, campagne trois lieux et références propres, signalisation privée et départ réussis. Ni microphones physiques ni trajet TURN réel testés par ce rapport.</x:v>
       </x:c>
       <x:c r="G16" s="12" t="str">
         <x:v>Un départ explicite retire le membre ; le transfert de responsable ne révèle pas les autres perceptions.</x:v>
@@ -17358,7 +17609,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra060023856a64296"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc35883761b6a46d2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17528,7 +17779,7 @@
         <x:v>Relâcher, perdre le focus, masquer la page, fermer la radio ou ouvrir une modale coupe la transmission.</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="40" customHeight="1">
+    <x:row r="9" ht="51" customHeight="1">
       <x:c r="A9" s="11" t="str">
         <x:v>R04</x:v>
       </x:c>
@@ -17536,7 +17787,7 @@
         <x:v>Sortie propre</x:v>
       </x:c>
       <x:c r="C9" s="11" t="str">
-        <x:v>Arrêter pistes, connexions et nœuds audio en quittant la salle.</x:v>
+        <x:v>Arrêter les pistes et connexions en quittant ; invalider aussi toute demande de microphone encore en attente.</x:v>
       </x:c>
       <x:c r="D9" s="11" t="str">
         <x:v>Aucun micro utilisé après sortie.</x:v>
@@ -17548,10 +17799,10 @@
         <x:v>Quitter / déconnecter</x:v>
       </x:c>
       <x:c r="G9" s="11" t="str">
-        <x:v>Indicateur micro navigateur s’éteint et le pair voit la déconnexion.</x:v>
+        <x:v>Un flux qui arrive après fermeture est arrêté immédiatement, sans être affecté à la radio.</x:v>
       </x:c>
       <x:c r="H9" s="11" t="str">
-        <x:v>Le test de code n’atteste pas encore le matériel physique.</x:v>
+        <x:v>La boîte de permission du navigateur peut répondre plus tard ; la protection porte sur le traitement du résultat. Matériel physique non éprouvé.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="51" customHeight="1">
@@ -18071,7 +18322,7 @@
         <x:v>Deux puis quatre microphones physiques, plusieurs navigateurs.</x:v>
       </x:c>
       <x:c r="H29" s="11" t="str">
-        <x:v>12 tests radio et négociation partielle dans deux onglets ne constituent pas un essai de microphones physiques ou d’écoute de flux vocal.</x:v>
+        <x:v>19 tests radio et la négociation partielle de la v0.2 ne constituent pas un essai de microphones physiques ou d’écoute de flux vocal.</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="40" customHeight="1">
@@ -18152,20 +18403,98 @@
         <x:v>Le test 1 / 2 / 3 est un autre appareil de preuve ; nommer le repère évite de comparer deux écrans différents.</x:v>
       </x:c>
     </x:row>
+    <x:row r="33" ht="40" customHeight="1">
+      <x:c r="A33" s="11" t="str">
+        <x:v>R28</x:v>
+      </x:c>
+      <x:c r="B33" s="11" t="str">
+        <x:v>Autorisation devenue obsolète</x:v>
+      </x:c>
+      <x:c r="C33" s="11" t="str">
+        <x:v>Éteindre le micro ou fermer la radio invalide la demande applicative encore en attente.</x:v>
+      </x:c>
+      <x:c r="D33" s="11" t="str">
+        <x:v>Si le navigateur fournit ensuite un flux, arrêter toutes ses pistes avant toute installation.</x:v>
+      </x:c>
+      <x:c r="E33" s="13" t="str">
+        <x:v>Implémenté — QA partielle</x:v>
+      </x:c>
+      <x:c r="F33" s="11" t="str">
+        <x:v>Désactiver / quitter pendant la permission</x:v>
+      </x:c>
+      <x:c r="G33" s="11" t="str">
+        <x:v>Aucun flux tardif n’est conservé ni ajouté aux pairs ; les pistes sont effectivement stoppées.</x:v>
+      </x:c>
+      <x:c r="H33" s="11" t="str">
+        <x:v>La boîte système n’est pas prétendue annulée. Tests de promesses différées et de pistes simulées, matériel encore à vérifier.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="40" customHeight="1">
+      <x:c r="A34" s="12" t="str">
+        <x:v>R29</x:v>
+      </x:c>
+      <x:c r="B34" s="12" t="str">
+        <x:v>Réactivation récente</x:v>
+      </x:c>
+      <x:c r="C34" s="12" t="str">
+        <x:v>Chaque activation possède un identifiant de demande ; seul le résultat de la demande courante peut être retenu.</x:v>
+      </x:c>
+      <x:c r="D34" s="12" t="str">
+        <x:v>Ancien succès ou ancien refus après une nouvelle activation : état récent préservé.</x:v>
+      </x:c>
+      <x:c r="E34" s="13" t="str">
+        <x:v>Implémenté — QA partielle</x:v>
+      </x:c>
+      <x:c r="F34" s="12" t="str">
+        <x:v>Désactiver puis réactiver</x:v>
+      </x:c>
+      <x:c r="G34" s="12" t="str">
+        <x:v>L’ancienne réponse ne remplace pas le nouveau flux et ne réaffiche pas une erreur périmée.</x:v>
+      </x:c>
+      <x:c r="H34" s="12" t="str">
+        <x:v>Distinguer arrêt et simple mute : une piste muette doit aussi être arrêtée si sa demande est obsolète.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="40" customHeight="1">
+      <x:c r="A35" s="11" t="str">
+        <x:v>R30</x:v>
+      </x:c>
+      <x:c r="B35" s="11" t="str">
+        <x:v>Commande libérée</x:v>
+      </x:c>
+      <x:c r="C35" s="11" t="str">
+        <x:v>L’extinction invalide aussi l’opération en cours dans le contrôleur de l’interface.</x:v>
+      </x:c>
+      <x:c r="D35" s="11" t="str">
+        <x:v>La commande redevient disponible sans attendre la fin de l’ancienne permission.</x:v>
+      </x:c>
+      <x:c r="E35" s="13" t="str">
+        <x:v>Implémenté — QA partielle</x:v>
+      </x:c>
+      <x:c r="F35" s="11" t="str">
+        <x:v>Éteindre puis réactiver la radio</x:v>
+      </x:c>
+      <x:c r="G35" s="11" t="str">
+        <x:v>Un ancien résultat ou finaliseur ne bloque ni ne déverrouille à tort la nouvelle opération.</x:v>
+      </x:c>
+      <x:c r="H35" s="11" t="str">
+        <x:v>Contrôleur testé séparément du client vocal ; ces tests ne sont pas un essai de permission sur microphone physique.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="E6:E32">
+  <x:conditionalFormatting sqref="E6:E35">
     <x:cfRule type="containsText" dxfId="9" priority="1" operator="containsText" text="Bloqué"/>
     <x:cfRule type="containsText" dxfId="10" priority="2" operator="containsText" text="Validé"/>
     <x:cfRule type="containsText" dxfId="11" priority="3" operator="containsText" text="Réussi"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="E6:E32">
+    <x:dataValidation type="list" sqref="E6:E35">
       <x:formula1>"Présent,Prévu,Implémenté — QA partielle,Validé,À vérifier,Conçu — non implémenté,Bloqué,Réussi,Partiel,À exécuter,À tester sur GPU,À tester sur appareils,Conception définie,Contrôle structurel partiel"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8fe229cd51ae43f6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d358a9cbaef4e53"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18816,7 +19145,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1c63dfd74794f13"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red0cdd15c5124224"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19036,7 +19365,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R914392a9ea5d43d7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a7ae2a3476c4be6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19684,7 +20013,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdbe884bdf9c74482"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2424c44b8c9c40f4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20328,7 +20657,7 @@
         <x:v>Hôtel : 196 580 triangles ; métro : 84 278 ; clinique : 107 032, effets cachés compris. Inspecteur articulé : 52 444 triangles. Six surfaces planaires, deux actives par lieu.</x:v>
       </x:c>
       <x:c r="D30" s="12" t="str">
-        <x:v>11 suites CPU réussies : données finies, normales, luminaires, 48 effets et raycasts, corps/reflets sans récursion, retard réel proche d’une seconde, traversée des trois lieux, relais, collision, qualité et nettoyage.</x:v>
+        <x:v>Preuves v0.2 conservées : 11 suites CPU réussies : données finies, normales, luminaires, 48 effets et raycasts, corps/reflets sans récursion, retard réel proche d’une seconde, traversée des trois lieux, relais, collision, qualité et nettoyage.</x:v>
       </x:c>
       <x:c r="E30" s="13" t="str">
         <x:v>Contrôle structurel partiel</x:v>
@@ -20560,7 +20889,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebe31c88376f4dfb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb908f5982fa1425a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>